<commit_message>
DataSet cut by time/ sample greedy fature selection
</commit_message>
<xml_diff>
--- a/log/test_data_cat_clean.xlsx
+++ b/log/test_data_cat_clean.xlsx
@@ -463,11 +463,11 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[1559, 1603, 1820, 1823, 1914, 2218, 2219, 2220, 2580, 2581, 2582, 2792, 2892, 2893, 2894]</t>
+          <t>[89, 496, 712, 1280, 813]</t>
         </is>
       </c>
     </row>
@@ -491,11 +491,11 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>57</v>
+        <v>10</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[1514, 1518, 1561, 1564, 1594, 1597, 1607, 1620, 1730, 1774, 1791, 1804, 1807, 1832, 1840, 1841, 1858, 1859, 1860, 1861, 1862, 1863, 1864, 1894, 1903, 1959, 2046, 2049, 2068, 2082, 2154, 2180, 2190, 2191, 2199, 2225, 2238, 2388, 2403, 2415, 2548, 2553, 2554, 2558, 2703, 2738, 2767, 2768, 2790, 2803, 2813, 2814, 2829, 2860, 2898, 2906, 2909]</t>
+          <t>[985, 1351, 1451, 911, 1217, 79, 1284, 53, 1012, 635]</t>
         </is>
       </c>
     </row>
@@ -519,11 +519,11 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>31</v>
+        <v>7</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[1526, 1540, 1557, 1560, 1811, 1835, 1838, 2020, 2091, 2095, 2101, 2104, 2127, 2136, 2144, 2192, 2265, 2473, 2476, 2477, 2482, 2567, 2580, 2719, 2727, 2754, 2772, 2779, 2784, 2875, 2893]</t>
+          <t>[1187, 638, 1417, 862, 704, 706, 1145]</t>
         </is>
       </c>
     </row>
@@ -543,11 +543,11 @@
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>53</v>
+        <v>8</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[1472, 1473, 1474, 1475, 1499, 1500, 1614, 1615, 1652, 1653, 1655, 1656, 1676, 1739, 1908, 1910, 1962, 1963, 1964, 1966, 1984, 2029, 2034, 2036, 2037, 2210, 2244, 2245, 2247, 2283, 2284, 2285, 2305, 2306, 2308, 2370, 2371, 2570, 2602, 2603, 2605, 2645, 2646, 2647, 2650, 2651, 2714, 2819, 2866, 2910, 2913, 2914, 2915]</t>
+          <t>[57, 1043, 76, 656, 960, 1359, 1237, 1161]</t>
         </is>
       </c>
     </row>
@@ -599,11 +599,11 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>[1474, 1475, 1654, 1655, 1656, 1657, 1658, 1659, 1765, 1906, 1965, 1966, 2285, 2650, 2651]</t>
+          <t>[1161]</t>
         </is>
       </c>
     </row>
@@ -627,11 +627,11 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>66</v>
+        <v>15</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>[1479, 1503, 1581, 1583, 1604, 1614, 1615, 1616, 1617, 1630, 1631, 1632, 1642, 1678, 1915, 1917, 1921, 1922, 1926, 1939, 1971, 1972, 2008, 2221, 2222, 2242, 2243, 2244, 2245, 2247, 2261, 2262, 2268, 2288, 2290, 2295, 2340, 2351, 2364, 2372, 2373, 2392, 2507, 2526, 2550, 2566, 2583, 2602, 2603, 2604, 2605, 2625, 2629, 2658, 2686, 2718, 2773, 2895, 2896, 2907, 2910, 2911, 2913, 2914, 2915, 2916]</t>
+          <t>[317, 1008, 1218, 516, 400, 1289, 645, 76, 731, 1061, 345, 1087, 1458, 1268, 615]</t>
         </is>
       </c>
     </row>
@@ -655,11 +655,11 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>43</v>
+        <v>8</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>[1524, 1528, 1557, 1571, 1572, 1591, 1687, 1714, 1730, 1780, 1825, 1931, 1932, 1984, 1987, 2087, 2093, 2102, 2107, 2110, 2129, 2191, 2198, 2201, 2204, 2216, 2311, 2350, 2399, 2405, 2431, 2465, 2467, 2552, 2584, 2637, 2733, 2806, 2817, 2860, 2881, 2893, 2918]</t>
+          <t>[1385, 1400, 414, 1285, 1284, 770, 1237, 706]</t>
         </is>
       </c>
     </row>
@@ -683,11 +683,11 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>218</v>
+        <v>49</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>[1461, 1462, 1470, 1471, 1510, 1511, 1512, 1513, 1514, 1515, 1516, 1517, 1518, 1519, 1520, 1521, 1522, 1523, 1524, 1525, 1526, 1527, 1528, 1529, 1530, 1625, 1626, 1648, 1649, 1650, 1651, 1660, 1752, 1753, 1756, 1757, 1758, 1759, 1760, 1761, 1762, 1763, 1764, 1765, 1766, 1767, 1768, 1769, 1770, 1771, 1772, 1773, 1774, 1775, 1776, 1777, 1778, 1779, 1780, 1781, 1791, 1792, 1793, 1794, 1795, 1796, 1797, 1798, 1799, 1800, 1801, 1802, 1803, 1804, 1805, 1959, 1960, 1961, 2047, 2048, 2049, 2051, 2052, 2053, 2055, 2056, 2057, 2058, 2059, 2060, 2061, 2062, 2063, 2064, 2065, 2066, 2067, 2068, 2073, 2074, 2075, 2076, 2077, 2078, 2079, 2080, 2081, 2082, 2083, 2084, 2085, 2252, 2278, 2279, 2280, 2281, 2282, 2286, 2387, 2388, 2389, 2390, 2391, 2392, 2393, 2394, 2395, 2396, 2397, 2398, 2402, 2403, 2404, 2405, 2406, 2407, 2408, 2409, 2410, 2411, 2412, 2413, 2414, 2415, 2416, 2417, 2418, 2419, 2420, 2421, 2424, 2425, 2428, 2429, 2430, 2431, 2432, 2433, 2434, 2435, 2436, 2437, 2438, 2615, 2616, 2617, 2618, 2619, 2641, 2642, 2649, 2721, 2722, 2723, 2724, 2725, 2726, 2727, 2728, 2729, 2730, 2731, 2732, 2733, 2734, 2735, 2736, 2737, 2738, 2739, 2740, 2741, 2742, 2743, 2744, 2745, 2746, 2747, 2748, 2749, 2750, 2751, 2752, 2753, 2755, 2757, 2761, 2762, 2763, 2764, 2765, 2766, 2767, 2768, 2769, 2770, 2771, 2772]</t>
+          <t>[1351, 871, 866, 854, 874, 1451, 1412, 606, 38, 295, 761, 374, 1065, 726, 1126, 348, 659, 100, 39, 911, 626, 906, 17, 370, 628, 369, 1251, 1358, 34, 1027, 1291, 533, 141, 231, 1459, 74, 172, 1300, 1234, 27, 616, 1095, 447, 649, 143, 325, 255, 67, 420]</t>
         </is>
       </c>
     </row>

</xml_diff>